<commit_message>
added labels to reaction pathways, added the figures to validation section (docx only)
</commit_message>
<xml_diff>
--- a/icfd2026/paper/figures/reac_pathway_aid.xlsx
+++ b/icfd2026/paper/figures/reac_pathway_aid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\arr\lab\presentations\icfd2026\paper\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C1F856-312A-43CA-8B22-9D0B84D9F4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625B6463-AEE7-4411-9A4C-45816820657C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{13970726-6CA0-4D06-A476-A656A11058CA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{13970726-6CA0-4D06-A476-A656A11058CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="41">
   <si>
     <t>nh3-&gt;nh2</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>h2-&gt;h</t>
-  </si>
-  <si>
-    <t>nh2-&gt;n2h3</t>
   </si>
   <si>
     <t>nh</t>
@@ -231,7 +228,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="60">
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -266,566 +263,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1159,7 +596,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3283EA79-3C91-424F-96E1-9983A360E255}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1178,7 +614,7 @@
         <v>3.6599000000000001E-4</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H1" s="1">
         <v>5.4003999999999999E-4</v>
@@ -1203,7 +639,7 @@
         <v>2.2141639999999997E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -1225,7 +661,7 @@
         <v>1.8665402519999996E-4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>2</v>
       </c>
@@ -1247,7 +683,7 @@
         <v>7.5281575999999997E-6</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>3</v>
       </c>
@@ -1288,7 +724,7 @@
         <v>2.16016E-5</v>
       </c>
     </row>
-    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -1310,7 +746,7 @@
         <v>5.2275871999999999E-6</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -1332,7 +768,7 @@
         <v>6.8440130000000015E-6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -1373,7 +809,7 @@
         <v>1.4581080000000002E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>2</v>
       </c>
@@ -1395,7 +831,7 @@
         <v>5.3075131200000004E-5</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>1</v>
       </c>
@@ -1417,7 +853,7 @@
         <v>6.9114319199999998E-5</v>
       </c>
     </row>
-    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>6</v>
       </c>
@@ -1458,7 +894,7 @@
         <v>2.0000000000000002E-5</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>2</v>
       </c>
@@ -1480,7 +916,7 @@
         <v>2.7029001999999997E-5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>1</v>
       </c>
@@ -1524,7 +960,7 @@
         <v>0.26500000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>11</v>
       </c>
@@ -1546,7 +982,7 @@
         <v>1.5531550399999998E-5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>13</v>
       </c>
@@ -1590,7 +1026,7 @@
         <v>4.3000000000000002E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>6</v>
       </c>
@@ -1612,7 +1048,7 @@
         <v>4.20799168E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>15</v>
       </c>
@@ -1656,7 +1092,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>2</v>
       </c>
@@ -1678,7 +1114,7 @@
         <v>2.2465663999999999E-5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>3</v>
       </c>
@@ -1700,7 +1136,7 @@
         <v>1.8901400000000002E-6</v>
       </c>
     </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>1</v>
       </c>
@@ -1738,7 +1174,7 @@
         <v>1E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>12</v>
       </c>
@@ -1756,7 +1192,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B29">
         <v>0.3</v>
@@ -1776,9 +1212,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C30" s="2">
         <v>1</v>
@@ -1788,7 +1224,7 @@
         <v>1.0979699999999999E-5</v>
       </c>
       <c r="F30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G30" s="3">
         <v>1</v>
@@ -1800,7 +1236,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31">
         <v>0.2</v>
@@ -1814,7 +1250,7 @@
         <v>2.5000000000000001E-4</v>
       </c>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>2</v>
       </c>
@@ -1830,7 +1266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>7</v>
       </c>
@@ -1848,7 +1284,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D34" s="1"/>
       <c r="F34">
@@ -1863,7 +1299,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D35" s="1"/>
       <c r="F35" t="s">
         <v>6</v>
@@ -1878,7 +1314,7 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B36">
         <v>0.3</v>
@@ -1896,9 +1332,9 @@
         <v>3.24024E-5</v>
       </c>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C37" s="2">
         <v>1</v>
@@ -1908,7 +1344,7 @@
         <v>1.0979699999999999E-5</v>
       </c>
       <c r="F37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G37" s="2">
         <v>0.68100000000000005</v>
@@ -1918,7 +1354,7 @@
         <v>2.2066034400000001E-5</v>
       </c>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
         <v>6</v>
       </c>
@@ -1930,7 +1366,6 @@
         <v>1.0044743999999999E-5</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>18</v>
@@ -1944,7 +1379,7 @@
       </c>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>2</v>
       </c>
@@ -1976,7 +1411,7 @@
         <v>2.16016E-5</v>
       </c>
     </row>
-    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>2</v>
       </c>
@@ -2017,7 +1452,7 @@
         <v>3.456256E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>1</v>
       </c>
@@ -2039,7 +1474,7 @@
         <v>2.3813603839999999E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>3</v>
       </c>
@@ -2063,7 +1498,7 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B47">
         <v>1.5</v>
@@ -2080,7 +1515,7 @@
         <v>1.08008E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>3</v>
       </c>
@@ -2104,7 +1539,7 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B49">
         <v>3.6</v>
@@ -2121,7 +1556,7 @@
         <v>1.5121119999999999E-4</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>13</v>
       </c>
@@ -2143,114 +1578,114 @@
         <v>5.2772708799999992E-5</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C51" s="2">
         <v>0.25800000000000001</v>
       </c>
       <c r="D51" s="1">
-        <f>C51*$D$49</f>
+        <f t="shared" ref="D51:D56" si="8">C51*$D$49</f>
         <v>3.3993151200000001E-5</v>
       </c>
       <c r="F51" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G51" s="3">
         <v>0.20699999999999999</v>
       </c>
       <c r="H51" s="1">
-        <f>G51*$D$49</f>
+        <f t="shared" ref="H51:H56" si="9">G51*$D$49</f>
         <v>2.7273574799999998E-5</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C52" s="2">
         <v>0.13900000000000001</v>
       </c>
       <c r="D52" s="1">
-        <f>C52*$D$49</f>
+        <f t="shared" si="8"/>
         <v>1.8314139600000001E-5</v>
       </c>
       <c r="F52" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G52" s="3">
         <v>4.8000000000000001E-2</v>
       </c>
       <c r="H52" s="1">
-        <f>G52*$D$49</f>
+        <f t="shared" si="9"/>
         <v>6.3243071999999996E-6</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C53" s="2">
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="D53" s="1">
-        <f>C53*$D$49</f>
+        <f t="shared" si="8"/>
         <v>1.30438836E-5</v>
       </c>
       <c r="F53" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G53" s="3">
         <v>0.17299999999999999</v>
       </c>
       <c r="H53" s="1">
-        <f>G53*$D$49</f>
+        <f t="shared" si="9"/>
         <v>2.2793857199999998E-5</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C54" s="2">
         <v>6.3E-2</v>
       </c>
       <c r="D54" s="1">
-        <f>C54*$D$49</f>
+        <f t="shared" si="8"/>
         <v>8.3006531999999996E-6</v>
       </c>
       <c r="F54" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G54" s="3">
         <v>0.158</v>
       </c>
       <c r="H54" s="1">
-        <f>G54*$D$49</f>
+        <f t="shared" si="9"/>
         <v>2.0817511199999998E-5</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C55" s="2">
         <v>4.2000000000000003E-2</v>
       </c>
       <c r="D55" s="1">
-        <f>C55*$D$49</f>
+        <f t="shared" si="8"/>
         <v>5.5337687999999998E-6</v>
       </c>
       <c r="F55" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H55" s="1">
-        <f>G55*$D$49</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>7</v>
       </c>
@@ -2258,7 +1693,7 @@
         <v>4.1000000000000002E-2</v>
       </c>
       <c r="D56" s="1">
-        <f>C56*$D$49</f>
+        <f t="shared" si="8"/>
         <v>5.4020124000000002E-6</v>
       </c>
       <c r="F56" t="s">
@@ -2268,13 +1703,13 @@
         <v>5.2999999999999999E-2</v>
       </c>
       <c r="H56" s="1">
-        <f>G56*$D$49</f>
+        <f t="shared" si="9"/>
         <v>6.983089199999999E-6</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B57">
         <v>5.8</v>
@@ -2291,7 +1726,7 @@
         <v>2.7542039999999999E-4</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>15</v>
       </c>
@@ -2313,7 +1748,7 @@
         <v>2.3934032759999999E-4</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>7</v>
       </c>
@@ -2321,7 +1756,7 @@
         <v>0.214</v>
       </c>
       <c r="D59" s="1">
-        <f t="shared" ref="D59:D61" si="8">C59*D$57</f>
+        <f t="shared" ref="D59:D61" si="10">C59*D$57</f>
         <v>4.5426678799999996E-5</v>
       </c>
       <c r="F59" t="s">
@@ -2331,57 +1766,57 @@
         <v>0.04</v>
       </c>
       <c r="H59" s="1">
-        <f t="shared" ref="H59:H61" si="9">G59*H$57</f>
+        <f t="shared" ref="H59:H61" si="11">G59*H$57</f>
         <v>1.1016816E-5</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C60" s="2">
         <v>7.5999999999999998E-2</v>
       </c>
       <c r="D60" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.6132839199999999E-5</v>
       </c>
       <c r="F60" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G60" s="3">
         <v>6.9000000000000006E-2</v>
       </c>
       <c r="H60" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>1.9004007600000002E-5</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C61" s="2">
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="D61" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>3.8209355999999997E-6</v>
       </c>
       <c r="F61" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G61" s="3">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="H61" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>4.1313059999999995E-6</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B62">
         <v>5.8</v>
@@ -2398,9 +1833,9 @@
         <v>2.592192E-4</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C63" s="2">
         <v>0.94299999999999995</v>
@@ -2410,7 +1845,7 @@
         <v>2.0017457059999999E-4</v>
       </c>
       <c r="F63" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G63" s="3">
         <v>0.91800000000000004</v>
@@ -2420,53 +1855,53 @@
         <v>2.379632256E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C64" s="2">
         <v>0.04</v>
       </c>
       <c r="D64" s="1">
-        <f t="shared" ref="D64:D65" si="10">C64*D$62</f>
+        <f t="shared" ref="D64:D65" si="12">C64*D$62</f>
         <v>8.4909679999999996E-6</v>
       </c>
       <c r="F64" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G64" s="3">
         <v>4.1000000000000002E-2</v>
       </c>
       <c r="H64" s="1">
-        <f t="shared" ref="H64:H65" si="11">G64*H$62</f>
+        <f t="shared" ref="H64:H65" si="13">G64*H$62</f>
         <v>1.06279872E-5</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C65" s="2">
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="D65" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3.6086614E-6</v>
       </c>
       <c r="F65" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G65" s="3">
         <v>4.1000000000000002E-2</v>
       </c>
       <c r="H65" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>1.06279872E-5</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B66">
         <v>10</v>
@@ -2483,9 +1918,9 @@
         <v>5.4003999999999999E-4</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C67" s="2">
         <v>0.54300000000000004</v>
@@ -2495,7 +1930,7 @@
         <v>1.9873257000000002E-4</v>
       </c>
       <c r="F67" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G67" s="3">
         <v>0.44</v>
@@ -2505,19 +1940,19 @@
         <v>2.3761759999999999E-4</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C68" s="2">
         <v>3.1099999999999999E-2</v>
       </c>
       <c r="D68" s="1">
-        <f t="shared" ref="D68:D74" si="12">C68*D$66</f>
+        <f t="shared" ref="D68:D74" si="14">C68*D$66</f>
         <v>1.1382288999999999E-5</v>
       </c>
       <c r="F68" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G68" s="3">
         <v>0.34200000000000003</v>
@@ -2527,7 +1962,7 @@
         <v>1.8469368000000001E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
         <v>13</v>
       </c>
@@ -2535,7 +1970,7 @@
         <v>6.2E-2</v>
       </c>
       <c r="D69" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>2.269138E-5</v>
       </c>
       <c r="F69" t="s">
@@ -2549,7 +1984,7 @@
         <v>6.9125119999999995E-5</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>12</v>
       </c>
@@ -2557,7 +1992,7 @@
         <v>0.02</v>
       </c>
       <c r="D70" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>7.3198000000000006E-6</v>
       </c>
       <c r="F70" t="s">
@@ -2571,19 +2006,19 @@
         <v>3.0242239999999999E-5</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C71" s="2">
         <v>1.6E-2</v>
       </c>
       <c r="D71" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>5.8558400000000002E-6</v>
       </c>
       <c r="F71" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G71" s="3">
         <v>1.9E-2</v>
@@ -2593,23 +2028,23 @@
         <v>1.0260759999999999E-5</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C72" s="2">
         <v>1.6E-2</v>
       </c>
       <c r="D72" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>5.8558400000000002E-6</v>
       </c>
       <c r="F72" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H72" s="1"/>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
         <v>7</v>
       </c>
@@ -2617,7 +2052,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
       <c r="D73" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>4.7578700000000002E-6</v>
       </c>
       <c r="F73" t="s">
@@ -2625,25 +2060,25 @@
       </c>
       <c r="H73" s="1"/>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C74" s="2">
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="D74" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>4.02589E-6</v>
       </c>
       <c r="F74" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H74" s="1"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B75">
         <v>2.9</v>
@@ -2660,7 +2095,7 @@
         <v>1.1340840000000001E-4</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>6</v>
       </c>
@@ -2898,31 +2333,25 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H76" xr:uid="{3283EA79-3C91-424F-96E1-9983A360E255}">
-    <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H76" xr:uid="{3283EA79-3C91-424F-96E1-9983A360E255}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D81:D118">
     <sortCondition ref="D81:D118"/>
   </sortState>
   <conditionalFormatting sqref="D2:D75 H2:H75">
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="between">
-      <formula>$J$14</formula>
-      <formula>$J$20</formula>
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+      <formula>$J$31</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
+      <formula>$J$27</formula>
+      <formula>$J$31</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="3" operator="between">
       <formula>$J$20</formula>
       <formula>$J$27</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
-      <formula>$J$27</formula>
-      <formula>$J$31</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
-      <formula>$J$31</formula>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="between">
+      <formula>$J$14</formula>
+      <formula>$J$20</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>